<commit_message>
Add NAV + FCF generated layer (forward NAV at end-2030)
Equity FCF 2027-2030 (asset margin + retail, less overhead, interest, cash tax,
preferred dividends) plus equity NAV of the remaining asset life at end-2030,
with implied annual return from today's price. Avoids double counting FCF that
today's NAV already includes; the naive sum is shown only for contrast.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012DJcvzRgw71v4Pt1pz75iK
</commit_message>
<xml_diff>
--- a/nav_model/outputs/nav_model.xlsx
+++ b/nav_model/outputs/nav_model.xlsx
@@ -18,6 +18,8 @@
     <sheet name="Revenue streams annual" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Claims" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="Asset register" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="NAV + FCF" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Equity FCF annual" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1324,7 +1326,6 @@
       <c r="G2" t="n">
         <v>2055</v>
       </c>
-      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1428,7 +1429,6 @@
       <c r="G5" t="n">
         <v>2055</v>
       </c>
-      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1460,7 +1460,6 @@
       <c r="G6" t="n">
         <v>2055</v>
       </c>
-      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1528,7 +1527,6 @@
       <c r="G8" t="n">
         <v>2055</v>
       </c>
-      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1554,7 +1552,6 @@
       <c r="E9" t="n">
         <v>1900</v>
       </c>
-      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1586,7 +1583,6 @@
       <c r="G10" t="n">
         <v>2050</v>
       </c>
-      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1618,7 +1614,6 @@
       <c r="G11" t="n">
         <v>2038</v>
       </c>
-      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1650,7 +1645,6 @@
       <c r="G12" t="n">
         <v>2038</v>
       </c>
-      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1682,7 +1676,6 @@
       <c r="G13" t="n">
         <v>2045</v>
       </c>
-      <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1714,7 +1707,6 @@
       <c r="G14" t="n">
         <v>2040</v>
       </c>
-      <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1746,7 +1738,6 @@
       <c r="G15" t="n">
         <v>2045</v>
       </c>
-      <c r="H15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1778,7 +1769,6 @@
       <c r="G16" t="n">
         <v>2040</v>
       </c>
-      <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1846,7 +1836,6 @@
       <c r="G18" t="n">
         <v>2045</v>
       </c>
-      <c r="H18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1878,7 +1867,6 @@
       <c r="G19" t="n">
         <v>2050</v>
       </c>
-      <c r="H19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1982,7 +1970,6 @@
       <c r="G22" t="n">
         <v>2055</v>
       </c>
-      <c r="H22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2014,7 +2001,6 @@
       <c r="G23" t="n">
         <v>2045</v>
       </c>
-      <c r="H23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2046,7 +2032,6 @@
       <c r="G24" t="n">
         <v>2040</v>
       </c>
-      <c r="H24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2078,7 +2063,6 @@
       <c r="G25" t="n">
         <v>2045</v>
       </c>
-      <c r="H25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2110,7 +2094,6 @@
       <c r="G26" t="n">
         <v>2045</v>
       </c>
-      <c r="H26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2142,7 +2125,6 @@
       <c r="G27" t="n">
         <v>2040</v>
       </c>
-      <c r="H27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2174,7 +2156,6 @@
       <c r="G28" t="n">
         <v>2038</v>
       </c>
-      <c r="H28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2206,7 +2187,6 @@
       <c r="G29" t="n">
         <v>2035</v>
       </c>
-      <c r="H29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2238,7 +2218,6 @@
       <c r="G30" t="n">
         <v>2027</v>
       </c>
-      <c r="H30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2264,7 +2243,6 @@
       <c r="E31" t="n">
         <v>1274</v>
       </c>
-      <c r="H31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2296,7 +2274,6 @@
       <c r="G32" t="n">
         <v>2050</v>
       </c>
-      <c r="H32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2328,7 +2305,1708 @@
       <c r="G33" t="n">
         <v>2050</v>
       </c>
-      <c r="H33" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>company</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>scenario</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>fcf27</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>yield27</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>cum_ps</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>fwd_ps</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>total_ps</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>irr</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>pv_total_ps</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>today_ps</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>naive_ps</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>CEG</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>7.9554</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.0851</v>
+      </c>
+      <c r="E2" t="n">
+        <v>72.6011</v>
+      </c>
+      <c r="F2" t="n">
+        <v>55.8617</v>
+      </c>
+      <c r="G2" t="n">
+        <v>128.4628</v>
+      </c>
+      <c r="H2" t="n">
+        <v>-0.1558</v>
+      </c>
+      <c r="I2" t="n">
+        <v>100.4862</v>
+      </c>
+      <c r="J2" t="n">
+        <v>93.6392</v>
+      </c>
+      <c r="K2" t="n">
+        <v>166.2403</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CEG</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>8.0281</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.0859</v>
+      </c>
+      <c r="E3" t="n">
+        <v>87.5294</v>
+      </c>
+      <c r="F3" t="n">
+        <v>174.9623</v>
+      </c>
+      <c r="G3" t="n">
+        <v>262.4916</v>
+      </c>
+      <c r="H3" t="n">
+        <v>-0.0013</v>
+      </c>
+      <c r="I3" t="n">
+        <v>194.2765</v>
+      </c>
+      <c r="J3" t="n">
+        <v>189.6628</v>
+      </c>
+      <c r="K3" t="n">
+        <v>277.1922</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>CEG</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>8.1008</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.0866</v>
+      </c>
+      <c r="E4" t="n">
+        <v>103.0812</v>
+      </c>
+      <c r="F4" t="n">
+        <v>295.4722</v>
+      </c>
+      <c r="G4" t="n">
+        <v>398.5533</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.1018</v>
+      </c>
+      <c r="I4" t="n">
+        <v>289.5044</v>
+      </c>
+      <c r="J4" t="n">
+        <v>287.0323</v>
+      </c>
+      <c r="K4" t="n">
+        <v>390.1134</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>CEG</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Extreme</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>8.189299999999999</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.0876</v>
+      </c>
+      <c r="E5" t="n">
+        <v>126.1365</v>
+      </c>
+      <c r="F5" t="n">
+        <v>474.4976</v>
+      </c>
+      <c r="G5" t="n">
+        <v>600.6342</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.2135</v>
+      </c>
+      <c r="I5" t="n">
+        <v>430.9156</v>
+      </c>
+      <c r="J5" t="n">
+        <v>431.5404</v>
+      </c>
+      <c r="K5" t="n">
+        <v>557.677</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>VST</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>5.8357</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.1233</v>
+      </c>
+      <c r="E6" t="n">
+        <v>48.1748</v>
+      </c>
+      <c r="F6" t="n">
+        <v>2.192</v>
+      </c>
+      <c r="G6" t="n">
+        <v>50.3668</v>
+      </c>
+      <c r="H6" t="n">
+        <v>-0.2122</v>
+      </c>
+      <c r="I6" t="n">
+        <v>42.7681</v>
+      </c>
+      <c r="J6" t="n">
+        <v>27.0779</v>
+      </c>
+      <c r="K6" t="n">
+        <v>75.25279999999999</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>VST</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>5.9059</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.1248</v>
+      </c>
+      <c r="E7" t="n">
+        <v>59.1173</v>
+      </c>
+      <c r="F7" t="n">
+        <v>70.46210000000001</v>
+      </c>
+      <c r="G7" t="n">
+        <v>129.5794</v>
+      </c>
+      <c r="H7" t="n">
+        <v>-0.016</v>
+      </c>
+      <c r="I7" t="n">
+        <v>98.3381</v>
+      </c>
+      <c r="J7" t="n">
+        <v>82.06619999999999</v>
+      </c>
+      <c r="K7" t="n">
+        <v>141.1835</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>VST</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>5.976</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.1263</v>
+      </c>
+      <c r="E8" t="n">
+        <v>71.1301</v>
+      </c>
+      <c r="F8" t="n">
+        <v>142.4178</v>
+      </c>
+      <c r="G8" t="n">
+        <v>213.5479</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.1068</v>
+      </c>
+      <c r="I8" t="n">
+        <v>157.2585</v>
+      </c>
+      <c r="J8" t="n">
+        <v>140.311</v>
+      </c>
+      <c r="K8" t="n">
+        <v>211.4411</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>VST</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Extreme</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>6.0615</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.1281</v>
+      </c>
+      <c r="E9" t="n">
+        <v>89.4744</v>
+      </c>
+      <c r="F9" t="n">
+        <v>252.5365</v>
+      </c>
+      <c r="G9" t="n">
+        <v>342.0109</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.2365</v>
+      </c>
+      <c r="I9" t="n">
+        <v>247.3764</v>
+      </c>
+      <c r="J9" t="n">
+        <v>229.3551</v>
+      </c>
+      <c r="K9" t="n">
+        <v>318.8295</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>company</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>scenario</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>revenue</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>asset_margin</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>platform</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>overhead</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>tax</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>pref</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>fcf</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>CEG</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D2" t="n">
+        <v>21.299</v>
+      </c>
+      <c r="E2" t="n">
+        <v>10.112</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.459</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.729</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1.989</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>7.955</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CEG</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>2028</v>
+      </c>
+      <c r="D3" t="n">
+        <v>22.286</v>
+      </c>
+      <c r="E3" t="n">
+        <v>11.095</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.468</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.729</v>
+      </c>
+      <c r="I3" t="n">
+        <v>2.188</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>8.750999999999999</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>CEG</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>2029</v>
+      </c>
+      <c r="D4" t="n">
+        <v>18.734</v>
+      </c>
+      <c r="E4" t="n">
+        <v>7.246</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1.061</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.478</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.729</v>
+      </c>
+      <c r="I4" t="n">
+        <v>1.415</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>5.686</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>CEG</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>2030</v>
+      </c>
+      <c r="D5" t="n">
+        <v>15.936</v>
+      </c>
+      <c r="E5" t="n">
+        <v>4.271</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1.082</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.487</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.729</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.806</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>3.331</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>CEG</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D6" t="n">
+        <v>21.384</v>
+      </c>
+      <c r="E6" t="n">
+        <v>10.203</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.459</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.729</v>
+      </c>
+      <c r="I6" t="n">
+        <v>2.007</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>8.028</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>CEG</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>2028</v>
+      </c>
+      <c r="D7" t="n">
+        <v>22.372</v>
+      </c>
+      <c r="E7" t="n">
+        <v>11.188</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.468</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.729</v>
+      </c>
+      <c r="I7" t="n">
+        <v>2.206</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>8.824999999999999</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>CEG</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>2029</v>
+      </c>
+      <c r="D8" t="n">
+        <v>21.049</v>
+      </c>
+      <c r="E8" t="n">
+        <v>9.541</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1.061</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.478</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.729</v>
+      </c>
+      <c r="I8" t="n">
+        <v>1.879</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>7.516</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>CEG</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>2030</v>
+      </c>
+      <c r="D9" t="n">
+        <v>20.214</v>
+      </c>
+      <c r="E9" t="n">
+        <v>8.436999999999999</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1.082</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.487</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.729</v>
+      </c>
+      <c r="I9" t="n">
+        <v>1.661</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
+        <v>6.643</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>CEG</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D10" t="n">
+        <v>21.468</v>
+      </c>
+      <c r="E10" t="n">
+        <v>10.294</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.459</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.729</v>
+      </c>
+      <c r="I10" t="n">
+        <v>2.025</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
+        <v>8.101000000000001</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>CEG</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>2028</v>
+      </c>
+      <c r="D11" t="n">
+        <v>22.458</v>
+      </c>
+      <c r="E11" t="n">
+        <v>11.281</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.468</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.729</v>
+      </c>
+      <c r="I11" t="n">
+        <v>2.225</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" t="n">
+        <v>8.898999999999999</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>CEG</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>2029</v>
+      </c>
+      <c r="D12" t="n">
+        <v>23.393</v>
+      </c>
+      <c r="E12" t="n">
+        <v>11.891</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1.061</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.478</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.729</v>
+      </c>
+      <c r="I12" t="n">
+        <v>2.349</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" t="n">
+        <v>9.396000000000001</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>CEG</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>2030</v>
+      </c>
+      <c r="D13" t="n">
+        <v>24.562</v>
+      </c>
+      <c r="E13" t="n">
+        <v>12.792</v>
+      </c>
+      <c r="F13" t="n">
+        <v>1.082</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.487</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.729</v>
+      </c>
+      <c r="I13" t="n">
+        <v>2.532</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" t="n">
+        <v>10.126</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>CEG</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Extreme</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D14" t="n">
+        <v>21.569</v>
+      </c>
+      <c r="E14" t="n">
+        <v>10.405</v>
+      </c>
+      <c r="F14" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.459</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.729</v>
+      </c>
+      <c r="I14" t="n">
+        <v>2.047</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" t="n">
+        <v>8.189</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>CEG</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Extreme</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>2028</v>
+      </c>
+      <c r="D15" t="n">
+        <v>22.562</v>
+      </c>
+      <c r="E15" t="n">
+        <v>11.393</v>
+      </c>
+      <c r="F15" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.468</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.729</v>
+      </c>
+      <c r="I15" t="n">
+        <v>2.247</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" t="n">
+        <v>8.989000000000001</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>CEG</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Extreme</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>2029</v>
+      </c>
+      <c r="D16" t="n">
+        <v>26.861</v>
+      </c>
+      <c r="E16" t="n">
+        <v>15.369</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1.061</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.478</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0.729</v>
+      </c>
+      <c r="I16" t="n">
+        <v>3.045</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" t="n">
+        <v>12.179</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>CEG</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Extreme</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>2030</v>
+      </c>
+      <c r="D17" t="n">
+        <v>31.062</v>
+      </c>
+      <c r="E17" t="n">
+        <v>19.301</v>
+      </c>
+      <c r="F17" t="n">
+        <v>1.082</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0.487</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0.729</v>
+      </c>
+      <c r="I17" t="n">
+        <v>3.834</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" t="n">
+        <v>15.334</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>VST</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D18" t="n">
+        <v>16.917</v>
+      </c>
+      <c r="E18" t="n">
+        <v>7.677</v>
+      </c>
+      <c r="F18" t="n">
+        <v>1.492</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.357</v>
+      </c>
+      <c r="H18" t="n">
+        <v>1.286</v>
+      </c>
+      <c r="I18" t="n">
+        <v>1.505</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0.186</v>
+      </c>
+      <c r="K18" t="n">
+        <v>5.836</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>VST</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>2028</v>
+      </c>
+      <c r="D19" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="E19" t="n">
+        <v>6.901</v>
+      </c>
+      <c r="F19" t="n">
+        <v>1.522</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.364</v>
+      </c>
+      <c r="H19" t="n">
+        <v>1.286</v>
+      </c>
+      <c r="I19" t="n">
+        <v>1.355</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0.186</v>
+      </c>
+      <c r="K19" t="n">
+        <v>5.233</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>VST</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>2029</v>
+      </c>
+      <c r="D20" t="n">
+        <v>13.301</v>
+      </c>
+      <c r="E20" t="n">
+        <v>4.467</v>
+      </c>
+      <c r="F20" t="n">
+        <v>1.553</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0.371</v>
+      </c>
+      <c r="H20" t="n">
+        <v>1.286</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0.864</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0.186</v>
+      </c>
+      <c r="K20" t="n">
+        <v>3.312</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>VST</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>2030</v>
+      </c>
+      <c r="D21" t="n">
+        <v>11.775</v>
+      </c>
+      <c r="E21" t="n">
+        <v>2.851</v>
+      </c>
+      <c r="F21" t="n">
+        <v>1.584</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="H21" t="n">
+        <v>1.286</v>
+      </c>
+      <c r="I21" t="n">
+        <v>0.537</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0.186</v>
+      </c>
+      <c r="K21" t="n">
+        <v>2.047</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>VST</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D22" t="n">
+        <v>16.998</v>
+      </c>
+      <c r="E22" t="n">
+        <v>7.765</v>
+      </c>
+      <c r="F22" t="n">
+        <v>1.492</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0.357</v>
+      </c>
+      <c r="H22" t="n">
+        <v>1.286</v>
+      </c>
+      <c r="I22" t="n">
+        <v>1.523</v>
+      </c>
+      <c r="J22" t="n">
+        <v>0.186</v>
+      </c>
+      <c r="K22" t="n">
+        <v>5.906</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>VST</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>2028</v>
+      </c>
+      <c r="D23" t="n">
+        <v>15.583</v>
+      </c>
+      <c r="E23" t="n">
+        <v>6.99</v>
+      </c>
+      <c r="F23" t="n">
+        <v>1.522</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0.364</v>
+      </c>
+      <c r="H23" t="n">
+        <v>1.286</v>
+      </c>
+      <c r="I23" t="n">
+        <v>1.373</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0.186</v>
+      </c>
+      <c r="K23" t="n">
+        <v>5.304</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>VST</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>2029</v>
+      </c>
+      <c r="D24" t="n">
+        <v>14.94</v>
+      </c>
+      <c r="E24" t="n">
+        <v>6.068</v>
+      </c>
+      <c r="F24" t="n">
+        <v>1.553</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0.371</v>
+      </c>
+      <c r="H24" t="n">
+        <v>1.286</v>
+      </c>
+      <c r="I24" t="n">
+        <v>1.193</v>
+      </c>
+      <c r="J24" t="n">
+        <v>0.186</v>
+      </c>
+      <c r="K24" t="n">
+        <v>4.585</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>VST</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>2030</v>
+      </c>
+      <c r="D25" t="n">
+        <v>14.829</v>
+      </c>
+      <c r="E25" t="n">
+        <v>5.768</v>
+      </c>
+      <c r="F25" t="n">
+        <v>1.584</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="H25" t="n">
+        <v>1.286</v>
+      </c>
+      <c r="I25" t="n">
+        <v>1.137</v>
+      </c>
+      <c r="J25" t="n">
+        <v>0.186</v>
+      </c>
+      <c r="K25" t="n">
+        <v>4.364</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>VST</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D26" t="n">
+        <v>17.079</v>
+      </c>
+      <c r="E26" t="n">
+        <v>7.853</v>
+      </c>
+      <c r="F26" t="n">
+        <v>1.492</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0.357</v>
+      </c>
+      <c r="H26" t="n">
+        <v>1.286</v>
+      </c>
+      <c r="I26" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="J26" t="n">
+        <v>0.186</v>
+      </c>
+      <c r="K26" t="n">
+        <v>5.976</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>VST</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>2028</v>
+      </c>
+      <c r="D27" t="n">
+        <v>15.666</v>
+      </c>
+      <c r="E27" t="n">
+        <v>7.08</v>
+      </c>
+      <c r="F27" t="n">
+        <v>1.522</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0.364</v>
+      </c>
+      <c r="H27" t="n">
+        <v>1.286</v>
+      </c>
+      <c r="I27" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="J27" t="n">
+        <v>0.186</v>
+      </c>
+      <c r="K27" t="n">
+        <v>5.376</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>VST</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>2029</v>
+      </c>
+      <c r="D28" t="n">
+        <v>16.658</v>
+      </c>
+      <c r="E28" t="n">
+        <v>7.793</v>
+      </c>
+      <c r="F28" t="n">
+        <v>1.553</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0.371</v>
+      </c>
+      <c r="H28" t="n">
+        <v>1.286</v>
+      </c>
+      <c r="I28" t="n">
+        <v>1.538</v>
+      </c>
+      <c r="J28" t="n">
+        <v>0.186</v>
+      </c>
+      <c r="K28" t="n">
+        <v>5.965</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>VST</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>2030</v>
+      </c>
+      <c r="D29" t="n">
+        <v>18.041</v>
+      </c>
+      <c r="E29" t="n">
+        <v>8.986000000000001</v>
+      </c>
+      <c r="F29" t="n">
+        <v>1.584</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="H29" t="n">
+        <v>1.286</v>
+      </c>
+      <c r="I29" t="n">
+        <v>1.781</v>
+      </c>
+      <c r="J29" t="n">
+        <v>0.186</v>
+      </c>
+      <c r="K29" t="n">
+        <v>6.939</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>VST</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Extreme</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D30" t="n">
+        <v>17.176</v>
+      </c>
+      <c r="E30" t="n">
+        <v>7.959</v>
+      </c>
+      <c r="F30" t="n">
+        <v>1.492</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0.357</v>
+      </c>
+      <c r="H30" t="n">
+        <v>1.286</v>
+      </c>
+      <c r="I30" t="n">
+        <v>1.562</v>
+      </c>
+      <c r="J30" t="n">
+        <v>0.186</v>
+      </c>
+      <c r="K30" t="n">
+        <v>6.061</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>VST</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Extreme</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>2028</v>
+      </c>
+      <c r="D31" t="n">
+        <v>15.765</v>
+      </c>
+      <c r="E31" t="n">
+        <v>7.189</v>
+      </c>
+      <c r="F31" t="n">
+        <v>1.522</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0.364</v>
+      </c>
+      <c r="H31" t="n">
+        <v>1.286</v>
+      </c>
+      <c r="I31" t="n">
+        <v>1.412</v>
+      </c>
+      <c r="J31" t="n">
+        <v>0.186</v>
+      </c>
+      <c r="K31" t="n">
+        <v>5.463</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>VST</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Extreme</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>2029</v>
+      </c>
+      <c r="D32" t="n">
+        <v>19.284</v>
+      </c>
+      <c r="E32" t="n">
+        <v>10.429</v>
+      </c>
+      <c r="F32" t="n">
+        <v>1.553</v>
+      </c>
+      <c r="G32" t="n">
+        <v>0.371</v>
+      </c>
+      <c r="H32" t="n">
+        <v>1.286</v>
+      </c>
+      <c r="I32" t="n">
+        <v>2.065</v>
+      </c>
+      <c r="J32" t="n">
+        <v>0.186</v>
+      </c>
+      <c r="K32" t="n">
+        <v>8.074</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>VST</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Extreme</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>2030</v>
+      </c>
+      <c r="D33" t="n">
+        <v>22.998</v>
+      </c>
+      <c r="E33" t="n">
+        <v>13.954</v>
+      </c>
+      <c r="F33" t="n">
+        <v>1.584</v>
+      </c>
+      <c r="G33" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="H33" t="n">
+        <v>1.286</v>
+      </c>
+      <c r="I33" t="n">
+        <v>2.774</v>
+      </c>
+      <c r="J33" t="n">
+        <v>0.186</v>
+      </c>
+      <c r="K33" t="n">
+        <v>10.912</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>